<commit_message>
map RWD and restructure home
</commit_message>
<xml_diff>
--- a/public/data/Taipei_Retro_Cafe.xlsx
+++ b/public/data/Taipei_Retro_Cafe.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="407">
   <si>
     <t>id</t>
   </si>
@@ -89,6 +89,9 @@
     <t>address_en</t>
   </si>
   <si>
+    <t>desc_en</t>
+  </si>
+  <si>
     <t>黑鳥咖啡</t>
   </si>
   <si>
@@ -128,6 +131,9 @@
     <t>No. 433, Zhonghe St, Beitou District</t>
   </si>
   <si>
+    <t>Named after the Beatles' classic song 'Blackbird,' this café is filled with Beatles memorabilia. In addition to freshly brewed espresso and hand-drip coffee, it offers a cozy space for the community to enjoy brunch or afternoon tea and savor life.</t>
+  </si>
+  <si>
     <t>皁咖啡</t>
   </si>
   <si>
@@ -152,6 +158,9 @@
     <t>2F, No. 3, Yuren Rd, Lane 8, Beitou District</t>
   </si>
   <si>
+    <t>Zao Café, tucked away in a quiet Beitou alley, blends local culture with modern style. Known for its hand-pour coffee and creative drinks, it offers a calm and stylish retreat from the city’s bustle.</t>
+  </si>
+  <si>
     <t>爐鍋咖啡</t>
   </si>
   <si>
@@ -176,6 +185,9 @@
     <t>No. 39, Lane 296, Section 3, Dadu Rd, Beitou District</t>
   </si>
   <si>
+    <t>Dedicated to sharing the beauty of coffee with friends, this café roasts its beans in-house and focuses on pure single-origin brews. Sugar and creamer are not provided, highlighting the coffee’s natural flavor.</t>
+  </si>
+  <si>
     <t>摩德年代</t>
   </si>
   <si>
@@ -212,6 +224,9 @@
     <t>No. 29, Lane 235, Zhongzheng Rd, Shilin District</t>
   </si>
   <si>
+    <t>A hidden late-night café near Shilin MRT, combining retro and industrial décor. It offers a variety of coffee and desserts in a relaxing environment, perfect for night owls seeking comfort.</t>
+  </si>
+  <si>
     <t>玄珠</t>
   </si>
   <si>
@@ -239,6 +254,9 @@
     <t>1F, No. 58, Zhongzheng Rd, Lane 213, Shilin District</t>
   </si>
   <si>
+    <t>Syuan Drew is a vintage-style café nestled in the alleys of Shilin. With carefully selected beans and a tranquil atmosphere, it offers a peaceful retreat for those who love both coffee and nostalgia.</t>
+  </si>
+  <si>
     <t>看電車咖啡</t>
   </si>
   <si>
@@ -266,6 +284,9 @@
     <t>No. 302, Wenlin Rd, Shilin District</t>
   </si>
   <si>
+    <t>Retro Station is a charming old-house café near Shipai Station. The warm vintage design, handcrafted lattes, and brunch options make it a great place to slow down and relax.</t>
+  </si>
+  <si>
     <t>幻猻家珈琲</t>
   </si>
   <si>
@@ -299,6 +320,9 @@
     <t>No. 14, Lane 14, Section 1, Dihua St, Datong District</t>
   </si>
   <si>
+    <t>With its nostalgic interior and relaxing vibe, this café offers hand-brewed coffee and a small selection of desserts. A perfect hideout to escape the city buzz.</t>
+  </si>
+  <si>
     <t>森高砂咖啡館</t>
   </si>
   <si>
@@ -320,6 +344,9 @@
     <t>No. 1, Section 2, Yanping N Rd, Datong District</t>
   </si>
   <si>
+    <t>A quiet corner in the neighborhood, offering rich espresso drinks and mellow music. The vintage furnishings and hand-pour brews create a comforting ambiance.</t>
+  </si>
+  <si>
     <t>TWATUTIA Coffee &amp; Co.</t>
   </si>
   <si>
@@ -344,6 +371,9 @@
     <t>No. 279, Nanjing W Rd, Datong District</t>
   </si>
   <si>
+    <t>This retro-themed café serves specialty hand-drip coffee and homemade desserts. Ideal for coffee lovers looking for a peaceful spot to read or work.</t>
+  </si>
+  <si>
     <t>PAI coffee</t>
   </si>
   <si>
@@ -377,6 +407,9 @@
     <t>No. 1, Alley 6, Lane 147, Section 2, Minsheng E Rd, Zhongshan District</t>
   </si>
   <si>
+    <t>Combining Taiwanese old-school charm with specialty brews, this café serves single-origin coffee in a cozy, low-key setting that invites you to linger.</t>
+  </si>
+  <si>
     <t>二會咖啡廳</t>
   </si>
   <si>
@@ -404,6 +437,9 @@
     <t>2F, No. 21, Huayin St, Zhongshan District</t>
   </si>
   <si>
+    <t>Tucked away in a quiet alley, this cozy café embraces a vintage atmosphere with warm wooden furnishings and soft lighting. It’s a go-to spot for hand-drip coffee lovers who enjoy tranquility. Whether you're here to read, work, or simply relax, the calm vibe invites you to stay. The baristas take pride in their craft, and the space feels like a quiet escape from the city.</t>
+  </si>
+  <si>
     <t>珈琲 寶山</t>
   </si>
   <si>
@@ -428,6 +464,9 @@
     <t>No. 36, Chang'an W Rd, Zhongshan District</t>
   </si>
   <si>
+    <t>Inspired by old-school aesthetics, this café mixes rustic wood décor with soft jazz in the background. Their hand-brewed coffee is the highlight, served with great attention to detail. Visitors can enjoy quiet corners, perfect for working or daydreaming. With natural light filtering through, it offers a peaceful oasis amidst the city buzz.</t>
+  </si>
+  <si>
     <t>Shawn</t>
   </si>
   <si>
@@ -452,6 +491,9 @@
     <t>No. 16, Lane 8, Xinzhong St, Songshan District</t>
   </si>
   <si>
+    <t>This café focuses on simplicity and warmth, inviting guests to take a break from the noise of everyday life. With retro-style furniture and soothing music, it’s a wonderful space to slow down. Their coffee is brewed with care and paired with light desserts. It’s ideal for solo visits or intimate conversations.</t>
+  </si>
+  <si>
     <t>民生工寓</t>
   </si>
   <si>
@@ -476,6 +518,9 @@
     <t>No. 3, Alley 1, Lane 56, Section 4, Minsheng E Rd, Songshan District</t>
   </si>
   <si>
+    <t>Located just minutes from the MRT, this café is a quiet sanctuary that blends retro charm with industrial accents. Inside, you’ll find carefully arranged vintage furniture and mellow lighting. Their pour-over coffee is rich and smooth, perfect for a relaxing afternoon. The vibe makes you want to linger just a bit longer.</t>
+  </si>
+  <si>
     <t>温咖啡</t>
   </si>
   <si>
@@ -503,6 +548,9 @@
     <t>No. 27, Lane 113, Section 3, Minsheng E Rd, Songshan District</t>
   </si>
   <si>
+    <t>Housed in a beautifully restored old building, this café celebrates nostalgia through its décor and ambiance. The interior showcases classic tiles, antique furniture, and thoughtful lighting. Hand-drip coffee and homemade desserts are the main attractions. Whether rain or shine, it’s a cozy corner to retreat into.</t>
+  </si>
+  <si>
     <t>自家屋珈琲焙煎所</t>
   </si>
   <si>
@@ -539,6 +587,9 @@
     <t>No. 2, Alley 4, Lane 437, Section 1, Neihu Rd, Neihu District</t>
   </si>
   <si>
+    <t>In this old-house café, every detail—from the wooden beams to the soft cushions—tells a story. You can enjoy slow mornings with a hot cup of pour-over coffee and a slice of cake. It's a favorite spot for artists, students, and coffee lovers. The homey feel makes it a memorable part of the neighborhood.</t>
+  </si>
+  <si>
     <t>河流咖啡</t>
   </si>
   <si>
@@ -560,6 +611,9 @@
     <t>No. 239, Section 2, Neihu Rd, Neihu District</t>
   </si>
   <si>
+    <t>Step into this café and be transported to a simpler time. The aroma of freshly ground beans greets you, accompanied by the gentle hum of vinyl records. Their specialty coffee is brewed with precision. The vintage surroundings create an atmosphere where time feels slower.</t>
+  </si>
+  <si>
     <t>TIECAFE</t>
   </si>
   <si>
@@ -581,6 +635,9 @@
     <t>1F, No. 56, Lane 426, Section 2, Chenggong Rd, Neihu District</t>
   </si>
   <si>
+    <t>This hidden gem is all about peaceful moments. From its old-school posters to handmade espresso drinks, every part is curated with care. Guests often spend hours reading or catching up with friends. It’s the kind of place where you feel instantly at home.</t>
+  </si>
+  <si>
     <t>月霞</t>
   </si>
   <si>
@@ -602,6 +659,9 @@
     <t>1F, No. 3, Lane 47, Chifeng St, Datong District</t>
   </si>
   <si>
+    <t>The café’s design nods to mid-century Taiwan, with classic tile patterns and antique touches. Hand-drip coffee is the star here, made with seasonal beans. The peaceful environment encourages thoughtful conversation. It’s a place where nostalgia and flavor meet.</t>
+  </si>
+  <si>
     <t>厝邊</t>
   </si>
   <si>
@@ -632,6 +692,9 @@
     <t>No. 12, Lane 20, Dali St, Wanhua District</t>
   </si>
   <si>
+    <t>Quietly located away from the main streets, this café is filled with natural light and old-world charm. The hand-brewed coffee is delicate and aromatic. With few seats and a slow pace, it’s perfect for introspective afternoons. You'll leave feeling both caffeinated and calm.</t>
+  </si>
+  <si>
     <t>町‧如固咖啡</t>
   </si>
   <si>
@@ -653,6 +716,9 @@
     <t>No. 113, Kunming St, Wanhua District</t>
   </si>
   <si>
+    <t>From its brick walls to its vintage teacups, this café delivers comfort and style. Pour-over coffee is prepared with attention and patience. It’s a haven for those seeking quiet joy and timeless surroundings. The peaceful rhythm of the space is instantly soothing.</t>
+  </si>
+  <si>
     <t>万 象</t>
   </si>
   <si>
@@ -686,6 +752,9 @@
     <t>No. 10, Lane 73, Tong'an St, Zhongzheng District</t>
   </si>
   <si>
+    <t>This small café packs a lot of character. Retro decor and warm smiles welcome you at the door. Their coffee is as rich in flavor as the space is in charm. It’s a space to sit back, sip slowly, and enjoy the moment.</t>
+  </si>
+  <si>
     <t>4F劇場咖啡</t>
   </si>
   <si>
@@ -704,6 +773,9 @@
     <t>4F, No. 98, Yanping S Rd, Zhongzheng District</t>
   </si>
   <si>
+    <t>Nestled in an old residential neighborhood, this café radiates warmth. The cozy layout encourages lingering. Each cup of coffee is brewed slowly, served with a smile. It’s the kind of spot you want to keep all to yourself.</t>
+  </si>
+  <si>
     <t>隅咖啡</t>
   </si>
   <si>
@@ -728,6 +800,9 @@
     <t>No. 175, Section 2, Tingzhou Rd, Zhongzheng District</t>
   </si>
   <si>
+    <t>Vintage lamps, hand-painted signage, and mellow tunes define the vibe here. The café’s staff are passionate about coffee, especially single-origin brews. The mix of nostalgia and refinement makes it special. It's both a retreat and an inspiration.</t>
+  </si>
+  <si>
     <t>Sugar Man Cafe</t>
   </si>
   <si>
@@ -758,6 +833,9 @@
     <t>No. 87-1, Section 1, Heping E Rd, Da’an District</t>
   </si>
   <si>
+    <t>This spot brings together old Taiwan aesthetics and modern café comfort. Expect hand-brewed coffee, soft lighting, and a peaceful vibe. The vintage interiors add depth and texture to your visit. Perfect for thoughtful breaks or casual hangs.</t>
+  </si>
+  <si>
     <t>秘式咖啡</t>
   </si>
   <si>
@@ -782,6 +860,9 @@
     <t>No. 30, Lane 4, Pucheng St, Da’an District</t>
   </si>
   <si>
+    <t>Old radios, floral tiles, and handcrafted lattes make this café one-of-a-kind. The balance of design and taste is deliberate. Their desserts complement the coffee perfectly. It's a sensory experience that blends past and present.</t>
+  </si>
+  <si>
     <t>翌日咖啡店</t>
   </si>
   <si>
@@ -809,6 +890,9 @@
     <t>No. 176, Chaozhou St, Da’an District</t>
   </si>
   <si>
+    <t>A small café with a big heart, this place is full of character. Antique decor lines the shelves, and the aroma of hand-pour coffee fills the air. It’s an inviting space where guests return again and again. The environment encourages genuine connection.</t>
+  </si>
+  <si>
     <t>James House</t>
   </si>
   <si>
@@ -827,6 +911,9 @@
     <t>1F, No. 1, Anhe Rd, Section 1, Lane 127, Alley 29, Da’an District</t>
   </si>
   <si>
+    <t>Designed for daydreaming, this café offers a quiet space for slow living. Wooden details, nostalgic music, and balanced brews define the experience. It’s the perfect place to read or simply watch the world go by. The calmness stays with you after you leave.</t>
+  </si>
+  <si>
     <t>50年代博物館咖啡</t>
   </si>
   <si>
@@ -860,6 +947,9 @@
     <t>No. 9-1, Lane 421, Guangfu S Rd, Xinyi District</t>
   </si>
   <si>
+    <t>This cozy nook embraces old-world style and hospitality. Guests are treated to finely brewed coffee and occasional homemade sweets. The lighting is gentle and the vibe unhurried. A true hideaway in the modern city.</t>
+  </si>
+  <si>
     <t>呷滴</t>
   </si>
   <si>
@@ -884,6 +974,9 @@
     <t>1F, No. 3, Alley 1, Lane 170, Wuxing St, Xinyi District</t>
   </si>
   <si>
+    <t>It’s more than a coffee stop—it’s a moment of pause. This retro-inspired space values quiet conversation and slow sips. From the tiles to the textures, every detail adds to the warmth. The coffee is smooth, the feeling sincere.</t>
+  </si>
+  <si>
     <t>Tropo Coffee</t>
   </si>
   <si>
@@ -908,6 +1001,9 @@
     <t>No. 49, Alley 22, Lane 553, Section 4, Zhongxiao E Rd, Xinyi District</t>
   </si>
   <si>
+    <t>A neighborhood favorite, this café charms with its antique décor and welcoming feel. The espresso is bold and thoughtfully made. The staff are kind and attentive. It’s a comforting place to land on any day.</t>
+  </si>
+  <si>
     <t>嘖咖啡</t>
   </si>
   <si>
@@ -938,6 +1034,9 @@
     <t>No. 135, Section 2, Nangang Rd, Nangang District</t>
   </si>
   <si>
+    <t>Housed in a narrow alley, this café feels like a secret worth sharing. Natural wood tones and old-world accents create intimacy. Their hand-drip coffee is nuanced and satisfying. A peaceful pocket tucked into the urban rush.</t>
+  </si>
+  <si>
     <t xml:space="preserve">玉虫画室 </t>
   </si>
   <si>
@@ -965,6 +1064,9 @@
     <t>No. 11, Lane 118, Section 2, Nangang Rd, Nangang District</t>
   </si>
   <si>
+    <t>The heart of this café lies in its love for storytelling—through both design and coffee. The vintage space invites you to slow down. Their brews are flavorful and grounded in care. You’ll want to stay longer than planned.</t>
+  </si>
+  <si>
     <t>田野咖啡</t>
   </si>
   <si>
@@ -992,6 +1094,9 @@
     <t>1F, No. 26, Lane 178, Section 2, Nangang Rd, Nangang District</t>
   </si>
   <si>
+    <t>Designed with a retro spirit, this café highlights Taiwan’s cultural past. The baristas are skilled in pour-over technique, and the drinks are beautifully balanced. It’s a space that feels both curated and homey.</t>
+  </si>
+  <si>
     <t>咖啡喫茶 枝音</t>
   </si>
   <si>
@@ -1028,6 +1133,9 @@
     <t>1F, No. 403, Section 3, Muxin Rd, Wenshan District</t>
   </si>
   <si>
+    <t>With antique chairs, framed maps, and wooden shelves, the space feels like a time capsule. Their coffee is brewed one cup at a time. Guests often come for the atmosphere and stay for the peace. It’s a gentle pause in your day.</t>
+  </si>
+  <si>
     <t>自由·之丘</t>
   </si>
   <si>
@@ -1049,6 +1157,9 @@
     <t>1F, No. 1, Lane 69, Section 2, Muxin Rd, Wenshan District</t>
   </si>
   <si>
+    <t>This space is a tribute to quiet beauty. Guests sip thoughtfully made drinks surrounded by retro details. It’s calm, familiar, and softly lit. The kind of place that becomes a habit.</t>
+  </si>
+  <si>
     <t>聞山咖啡</t>
   </si>
   <si>
@@ -1071,6 +1182,9 @@
   </si>
   <si>
     <t>No. 19, Jingzhong St, Wenshan District</t>
+  </si>
+  <si>
+    <t>Sunlight spills over the vintage tiles and weathered wood of this serene café. Their coffee is balanced and aromatic. Time seems to move differently here. Every visit feels like a treat.</t>
   </si>
   <si>
     <t>地區</t>
@@ -1185,7 +1299,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1203,6 +1317,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
@@ -1539,7 +1656,9 @@
       <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2"/>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="AA1" s="2"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="2"/>
@@ -1554,47 +1673,47 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q2" s="2">
         <v>25.1454118257922</v>
@@ -1603,27 +1722,29 @@
         <v>121.497706311702</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="V2" s="1">
         <v>4.9</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X2" s="1">
         <v>3.0</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z2" s="2"/>
+        <v>38</v>
+      </c>
+      <c r="Z2" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="AA2" s="2"/>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -1634,47 +1755,47 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="6">
+      <c r="A3" s="7">
         <v>2.0</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>39</v>
+      <c r="B3" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="Q3" s="2">
         <v>25.1337239581041</v>
@@ -1683,27 +1804,29 @@
         <v>121.498467604812</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="V3" s="1">
         <v>5.0</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X3" s="1">
         <v>6.0</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z3" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="Z3" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
@@ -1717,44 +1840,44 @@
       <c r="A4" s="1">
         <v>3.0</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>47</v>
+      <c r="B4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>50</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="Q4" s="2">
         <v>25.126614282379</v>
@@ -1763,27 +1886,29 @@
         <v>121.46776496189</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V4" s="1">
         <v>4.1</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X4" s="1">
         <v>6.0</v>
       </c>
       <c r="Y4" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z4" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="Z4" s="6" t="s">
+        <v>57</v>
+      </c>
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
@@ -1794,53 +1919,53 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="6">
+      <c r="A5" s="7">
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="Q5" s="2">
         <v>25.0947922353221</v>
@@ -1849,27 +1974,29 @@
         <v>121.526238028835</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="V5" s="1">
         <v>4.6</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="X5" s="1">
         <v>3.0</v>
       </c>
       <c r="Y5" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="Z5" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="Z5" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
       <c r="AC5" s="2"/>
@@ -1884,45 +2011,45 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>67</v>
+        <v>71</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="Q6" s="2">
         <v>25.0937038633108</v>
@@ -1931,27 +2058,29 @@
         <v>121.526950688694</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="T6" s="8" t="s">
-        <v>72</v>
+        <v>76</v>
+      </c>
+      <c r="T6" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="V6" s="1">
         <v>4.6</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="X6" s="1">
         <v>6.0</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="Z6" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Z6" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="2"/>
@@ -1962,51 +2091,51 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="6">
+      <c r="A7" s="7">
         <v>6.0</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>76</v>
+      <c r="B7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>82</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="Q7" s="2">
         <v>25.0920589737905</v>
@@ -2015,27 +2144,29 @@
         <v>121.526364995977</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="V7" s="1">
         <v>4.1</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="X7" s="1">
         <v>5.0</v>
       </c>
       <c r="Y7" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="Z7" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="Z7" s="6" t="s">
+        <v>90</v>
+      </c>
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
@@ -2050,44 +2181,44 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="Q8" s="2">
         <v>25.0543445672657</v>
@@ -2096,77 +2227,79 @@
         <v>121.509798373011</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="V8" s="1">
         <v>4.5</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="X8" s="1">
         <v>6.0</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="Z8" s="2"/>
+        <v>101</v>
+      </c>
+      <c r="Z8" s="6" t="s">
+        <v>102</v>
+      </c>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="6">
+      <c r="A9" s="7">
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="Q9" s="2">
         <v>25.055421878122</v>
@@ -2175,25 +2308,28 @@
         <v>121.511856896856</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="V9" s="1">
         <v>4.3</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="X9" s="1">
         <v>4.0</v>
       </c>
       <c r="Y9" s="5" t="s">
-        <v>101</v>
+        <v>109</v>
+      </c>
+      <c r="Z9" s="6" t="s">
+        <v>110</v>
       </c>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
@@ -2203,47 +2339,47 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="Q10" s="2">
         <v>25.053718503935</v>
@@ -2252,79 +2388,81 @@
         <v>121.509423901633</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="V10" s="1">
         <v>4.5</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="X10" s="1">
         <v>7.0</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="Z10" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="Z10" s="6" t="s">
+        <v>119</v>
+      </c>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="6">
+      <c r="A11" s="7">
         <v>10.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="Q11" s="2">
         <v>25.05929</v>
@@ -2333,27 +2471,29 @@
         <v>121.534699</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="T11" s="8" t="s">
-        <v>117</v>
+        <v>126</v>
+      </c>
+      <c r="T11" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="V11" s="1">
         <v>4.8</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="X11" s="1">
         <v>4.0</v>
       </c>
       <c r="Y11" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="Z11" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="Z11" s="6" t="s">
+        <v>131</v>
+      </c>
       <c r="AA11" s="2"/>
       <c r="AB11" s="2"/>
       <c r="AC11" s="2"/>
@@ -2363,49 +2503,49 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="Q12" s="2">
         <v>25.0494711344694</v>
@@ -2414,76 +2554,78 @@
         <v>121.520403595842</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="T12" s="8" t="s">
-        <v>127</v>
+        <v>137</v>
+      </c>
+      <c r="T12" s="9" t="s">
+        <v>138</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="V12" s="1">
         <v>4.5</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="X12" s="1">
         <v>5.0</v>
       </c>
       <c r="Y12" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="Z12" s="2"/>
+        <v>140</v>
+      </c>
+      <c r="Z12" s="6" t="s">
+        <v>141</v>
+      </c>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="6">
+      <c r="A13" s="7">
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="Q13" s="2">
         <v>25.0502418037303</v>
@@ -2492,27 +2634,29 @@
         <v>121.520509671541</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="T13" s="8" t="s">
-        <v>136</v>
+        <v>147</v>
+      </c>
+      <c r="T13" s="9" t="s">
+        <v>148</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="V13" s="1">
         <v>4.7</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="X13" s="1">
         <v>4.0</v>
       </c>
       <c r="Y13" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="Z13" s="2"/>
+        <v>149</v>
+      </c>
+      <c r="Z13" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="AA13" s="2"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
@@ -2522,49 +2666,49 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="Q14" s="2">
         <v>25.0597064867932</v>
@@ -2573,78 +2717,80 @@
         <v>121.561332665427</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="T14" s="8" t="s">
-        <v>143</v>
+        <v>155</v>
+      </c>
+      <c r="T14" s="9" t="s">
+        <v>156</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="V14" s="1">
         <v>4.6</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="X14" s="1">
         <v>3.0</v>
       </c>
       <c r="Y14" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z14" s="2"/>
+        <v>158</v>
+      </c>
+      <c r="Z14" s="6" t="s">
+        <v>159</v>
+      </c>
       <c r="AB14" s="2"/>
       <c r="AC14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="6">
+      <c r="A15" s="7">
         <v>14.0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="Q15" s="2">
         <v>25.0577731239708</v>
@@ -2653,27 +2799,29 @@
         <v>121.551858915285</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="T15" s="8" t="s">
-        <v>152</v>
+        <v>165</v>
+      </c>
+      <c r="T15" s="9" t="s">
+        <v>166</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="V15" s="1">
         <v>4.4</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="X15" s="1">
         <v>3.0</v>
       </c>
       <c r="Y15" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="Z15" s="2"/>
+        <v>167</v>
+      </c>
+      <c r="Z15" s="6" t="s">
+        <v>168</v>
+      </c>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
       <c r="AC15" s="2"/>
@@ -2683,45 +2831,45 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="Q16" s="2">
         <v>25.0602016716895</v>
@@ -2730,72 +2878,74 @@
         <v>121.546224411582</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="T16" s="3" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="V16" s="1">
         <v>4.5</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="X16" s="1">
         <v>3.0</v>
       </c>
       <c r="Y16" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="Z16" s="2"/>
+        <v>177</v>
+      </c>
+      <c r="Z16" s="6" t="s">
+        <v>178</v>
+      </c>
       <c r="AA16" s="2"/>
       <c r="AB16" s="2"/>
       <c r="AC16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="6">
+      <c r="A17" s="7">
         <v>16.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="J17" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="Q17" s="2">
         <v>25.0817588786275</v>
@@ -2804,27 +2954,29 @@
         <v>121.572125777881</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="T17" s="8" t="s">
-        <v>171</v>
+        <v>186</v>
+      </c>
+      <c r="T17" s="9" t="s">
+        <v>187</v>
       </c>
       <c r="U17" s="1" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="V17" s="1">
         <v>4.6</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="X17" s="1">
         <v>3.0</v>
       </c>
       <c r="Y17" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z17" s="2"/>
+        <v>190</v>
+      </c>
+      <c r="Z17" s="6" t="s">
+        <v>191</v>
+      </c>
       <c r="AA17" s="2"/>
       <c r="AB17" s="2"/>
       <c r="AC17" s="2"/>
@@ -2834,47 +2986,47 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="Q18" s="1">
         <v>25.0828824782301</v>
@@ -2883,79 +3035,81 @@
         <v>121.591301874655</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="T18" s="8" t="s">
-        <v>180</v>
+        <v>196</v>
+      </c>
+      <c r="T18" s="9" t="s">
+        <v>197</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="V18" s="1">
         <v>4.8</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="X18" s="1">
         <v>3.0</v>
       </c>
       <c r="Y18" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="Z18" s="2"/>
+        <v>198</v>
+      </c>
+      <c r="Z18" s="6" t="s">
+        <v>199</v>
+      </c>
       <c r="AA18" s="2"/>
       <c r="AB18" s="2"/>
       <c r="AC18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="6">
+      <c r="A19" s="7">
         <v>18.0</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
       <c r="Q19" s="1">
         <v>25.0708908180999</v>
@@ -2964,27 +3118,29 @@
         <v>121.590310021686</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="T19" s="8" t="s">
-        <v>187</v>
+        <v>204</v>
+      </c>
+      <c r="T19" s="9" t="s">
+        <v>205</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="V19" s="1">
         <v>4.6</v>
       </c>
       <c r="W19" s="1" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="X19" s="1">
         <v>3.0</v>
       </c>
       <c r="Y19" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="Z19" s="2"/>
+        <v>206</v>
+      </c>
+      <c r="Z19" s="6" t="s">
+        <v>207</v>
+      </c>
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
       <c r="AC19" s="2"/>
@@ -2994,49 +3150,49 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="Q20" s="2">
         <v>25.0555790808547</v>
@@ -3045,78 +3201,80 @@
         <v>121.519770028835</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="T20" s="8" t="s">
-        <v>194</v>
+        <v>212</v>
+      </c>
+      <c r="T20" s="9" t="s">
+        <v>213</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="V20" s="1">
         <v>4.4</v>
       </c>
       <c r="W20" s="1" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="X20" s="1">
         <v>3.0</v>
       </c>
       <c r="Y20" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="Z20" s="2"/>
+        <v>214</v>
+      </c>
+      <c r="Z20" s="6" t="s">
+        <v>215</v>
+      </c>
       <c r="AB20" s="2"/>
       <c r="AC20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="6">
+      <c r="A21" s="7">
         <v>20.0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>196</v>
+        <v>216</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="Q21" s="2">
         <v>25.0340065849163</v>
@@ -3125,27 +3283,29 @@
         <v>121.50214997574</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="T21" s="8" t="s">
-        <v>203</v>
+        <v>222</v>
+      </c>
+      <c r="T21" s="9" t="s">
+        <v>223</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="V21" s="1">
         <v>4.8</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>204</v>
+        <v>224</v>
       </c>
       <c r="X21" s="1">
         <v>3.0</v>
       </c>
       <c r="Y21" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="Z21" s="2"/>
+        <v>225</v>
+      </c>
+      <c r="Z21" s="6" t="s">
+        <v>226</v>
+      </c>
       <c r="AA21" s="2"/>
       <c r="AB21" s="2"/>
       <c r="AC21" s="2"/>
@@ -3154,47 +3314,47 @@
       <c r="A22" s="1">
         <v>21.0</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>207</v>
+      <c r="B22" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>228</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="Q22" s="2">
         <v>25.042256946363</v>
@@ -3203,76 +3363,78 @@
         <v>121.504808905538</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="T22" s="8" t="s">
-        <v>211</v>
+        <v>231</v>
+      </c>
+      <c r="T22" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="U22" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="V22" s="1">
         <v>4.3</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>204</v>
+        <v>224</v>
       </c>
       <c r="X22" s="1">
         <v>4.0</v>
       </c>
       <c r="Y22" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="Z22" s="2"/>
+        <v>233</v>
+      </c>
+      <c r="Z22" s="6" t="s">
+        <v>234</v>
+      </c>
       <c r="AA22" s="2"/>
       <c r="AB22" s="2"/>
       <c r="AC22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="6">
+      <c r="A23" s="7">
         <v>22.0</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
       <c r="Q23" s="2">
         <v>25.0234558406401</v>
@@ -3281,27 +3443,29 @@
         <v>121.521608432527</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="T23" s="9" t="s">
-        <v>220</v>
+        <v>241</v>
+      </c>
+      <c r="T23" s="10" t="s">
+        <v>242</v>
       </c>
       <c r="U23" s="1" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
       <c r="V23" s="1">
         <v>4.3</v>
       </c>
       <c r="W23" s="1" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="X23" s="1">
         <v>3.0</v>
       </c>
       <c r="Y23" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="Z23" s="2"/>
+        <v>245</v>
+      </c>
+      <c r="Z23" s="6" t="s">
+        <v>246</v>
+      </c>
       <c r="AB23" s="2"/>
       <c r="AC23" s="2"/>
     </row>
@@ -3309,50 +3473,50 @@
       <c r="A24" s="1">
         <v>23.0</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>225</v>
+      <c r="B24" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>248</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>226</v>
+        <v>249</v>
       </c>
       <c r="Q24" s="2">
         <v>25.0432120897679</v>
@@ -3361,72 +3525,74 @@
         <v>121.510247355253</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="T24" s="10" t="s">
-        <v>228</v>
+        <v>250</v>
+      </c>
+      <c r="T24" s="11" t="s">
+        <v>251</v>
       </c>
       <c r="U24" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="V24" s="1">
         <v>4.5</v>
       </c>
       <c r="W24" s="1" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="X24" s="1">
         <v>3.0</v>
       </c>
       <c r="Y24" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="Z24" s="2"/>
+        <v>252</v>
+      </c>
+      <c r="Z24" s="6" t="s">
+        <v>253</v>
+      </c>
       <c r="AA24" s="2"/>
       <c r="AB24" s="2"/>
       <c r="AC24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="6">
+      <c r="A25" s="7">
         <v>24.0</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>230</v>
+        <v>254</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>231</v>
+        <v>255</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="1" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>233</v>
+        <v>257</v>
       </c>
       <c r="Q25" s="2">
         <v>25.0245378348308</v>
@@ -3435,27 +3601,29 @@
         <v>121.521506273843</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="T25" s="11" t="s">
-        <v>235</v>
+        <v>258</v>
+      </c>
+      <c r="T25" s="12" t="s">
+        <v>259</v>
       </c>
       <c r="U25" s="1" t="s">
-        <v>236</v>
+        <v>260</v>
       </c>
       <c r="V25" s="1">
         <v>4.8</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="X25" s="1">
         <v>3.0</v>
       </c>
       <c r="Y25" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="Z25" s="2"/>
+        <v>261</v>
+      </c>
+      <c r="Z25" s="6" t="s">
+        <v>262</v>
+      </c>
       <c r="AA25" s="2"/>
       <c r="AB25" s="2"/>
       <c r="AC25" s="2"/>
@@ -3465,47 +3633,47 @@
         <v>25.0</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>238</v>
+        <v>263</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>238</v>
+        <v>263</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>239</v>
+        <v>264</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>240</v>
+        <v>265</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>242</v>
+        <v>267</v>
       </c>
       <c r="Q26" s="2">
         <v>25.0274227862327</v>
@@ -3514,74 +3682,76 @@
         <v>121.525673718276</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="T26" s="10" t="s">
-        <v>244</v>
+        <v>268</v>
+      </c>
+      <c r="T26" s="11" t="s">
+        <v>269</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>245</v>
+        <v>270</v>
       </c>
       <c r="V26" s="1">
         <v>3.8</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="X26" s="1">
         <v>3.0</v>
       </c>
       <c r="Y26" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="Z26" s="2"/>
+        <v>272</v>
+      </c>
+      <c r="Z26" s="6" t="s">
+        <v>273</v>
+      </c>
       <c r="AA26" s="2"/>
       <c r="AB26" s="2"/>
       <c r="AC26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="6">
+      <c r="A27" s="7">
         <v>26.0</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>248</v>
+        <v>274</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>239</v>
+        <v>264</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="Q27" s="2">
         <v>25.0246842675083</v>
@@ -3590,27 +3760,29 @@
         <v>121.525372771945</v>
       </c>
       <c r="S27" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="T27" s="9" t="s">
-        <v>253</v>
+        <v>278</v>
+      </c>
+      <c r="T27" s="10" t="s">
+        <v>279</v>
       </c>
       <c r="U27" s="1" t="s">
-        <v>254</v>
+        <v>280</v>
       </c>
       <c r="V27" s="1">
         <v>4.6</v>
       </c>
       <c r="W27" s="1" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="X27" s="1">
         <v>3.0</v>
       </c>
       <c r="Y27" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="Z27" s="2"/>
+        <v>281</v>
+      </c>
+      <c r="Z27" s="6" t="s">
+        <v>282</v>
+      </c>
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
       <c r="AC27" s="2"/>
@@ -3620,47 +3792,47 @@
         <v>27.0</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>239</v>
+        <v>264</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>258</v>
+        <v>285</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>260</v>
+        <v>287</v>
       </c>
       <c r="Q28" s="1">
         <v>25.0284375779507</v>
@@ -3669,77 +3841,79 @@
         <v>121.530202611108</v>
       </c>
       <c r="S28" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="T28" s="11" t="s">
-        <v>262</v>
+        <v>288</v>
+      </c>
+      <c r="T28" s="12" t="s">
+        <v>289</v>
       </c>
       <c r="U28" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="V28" s="1">
         <v>4.6</v>
       </c>
       <c r="W28" s="1" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="X28" s="1">
         <v>4.0</v>
       </c>
       <c r="Y28" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="Z28" s="2"/>
+        <v>291</v>
+      </c>
+      <c r="Z28" s="6" t="s">
+        <v>292</v>
+      </c>
       <c r="AA28" s="2"/>
       <c r="AB28" s="2"/>
       <c r="AC28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="6">
+      <c r="A29" s="7">
         <v>28.0</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>265</v>
+        <v>293</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>265</v>
+        <v>293</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>239</v>
+        <v>264</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>267</v>
+        <v>295</v>
       </c>
       <c r="Q29" s="1">
         <v>25.0354117110862</v>
@@ -3747,28 +3921,30 @@
       <c r="R29" s="1">
         <v>121.553897808577</v>
       </c>
-      <c r="S29" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="T29" s="8" t="s">
-        <v>269</v>
+      <c r="S29" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="T29" s="9" t="s">
+        <v>297</v>
       </c>
       <c r="U29" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="V29" s="1">
         <v>4.6</v>
       </c>
       <c r="W29" s="1" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="X29" s="1">
         <v>3.0</v>
       </c>
       <c r="Y29" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="Z29" s="2"/>
+        <v>298</v>
+      </c>
+      <c r="Z29" s="6" t="s">
+        <v>299</v>
+      </c>
       <c r="AA29" s="2"/>
       <c r="AB29" s="2"/>
       <c r="AC29" s="2"/>
@@ -3778,44 +3954,44 @@
         <v>29.0</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>274</v>
+        <v>303</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="Q30" s="2">
         <v>25.048715019923</v>
@@ -3824,77 +4000,79 @@
         <v>121.558957027833</v>
       </c>
       <c r="S30" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="T30" s="8" t="s">
-        <v>278</v>
+        <v>306</v>
+      </c>
+      <c r="T30" s="9" t="s">
+        <v>307</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>279</v>
+        <v>308</v>
       </c>
       <c r="V30" s="1">
         <v>4.7</v>
       </c>
       <c r="W30" s="1" t="s">
-        <v>280</v>
+        <v>309</v>
       </c>
       <c r="X30" s="1">
         <v>3.0</v>
       </c>
       <c r="Y30" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="Z30" s="2"/>
+        <v>310</v>
+      </c>
+      <c r="Z30" s="6" t="s">
+        <v>311</v>
+      </c>
       <c r="AA30" s="2"/>
       <c r="AB30" s="2"/>
       <c r="AC30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="6">
+      <c r="A31" s="7">
         <v>30.0</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>282</v>
+        <v>312</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>283</v>
+        <v>313</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>285</v>
+        <v>315</v>
       </c>
       <c r="Q31" s="2">
         <v>25.029759010615</v>
@@ -3902,26 +4080,29 @@
       <c r="R31" s="2">
         <v>121.563086959166</v>
       </c>
-      <c r="S31" s="12" t="s">
-        <v>286</v>
-      </c>
-      <c r="T31" s="8" t="s">
-        <v>287</v>
+      <c r="S31" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="T31" s="9" t="s">
+        <v>317</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>288</v>
+        <v>318</v>
       </c>
       <c r="V31" s="1">
         <v>4.5</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>280</v>
+        <v>309</v>
       </c>
       <c r="X31" s="1">
         <v>4.0</v>
       </c>
       <c r="Y31" s="1" t="s">
-        <v>289</v>
+        <v>319</v>
+      </c>
+      <c r="Z31" s="6" t="s">
+        <v>320</v>
       </c>
       <c r="AB31" s="2"/>
       <c r="AC31" s="2"/>
@@ -3931,45 +4112,45 @@
         <v>31.0</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>291</v>
+        <v>322</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="J32" s="1"/>
       <c r="K32" s="1" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="M32" s="1"/>
       <c r="N32" s="1" t="s">
-        <v>293</v>
+        <v>324</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
       <c r="Q32" s="1">
         <v>25.0437311273677</v>
@@ -3977,109 +4158,113 @@
       <c r="R32" s="1">
         <v>121.563566049973</v>
       </c>
-      <c r="S32" s="12" t="s">
-        <v>295</v>
-      </c>
-      <c r="T32" s="8" t="s">
-        <v>296</v>
+      <c r="S32" s="13" t="s">
+        <v>326</v>
+      </c>
+      <c r="T32" s="9" t="s">
+        <v>327</v>
       </c>
       <c r="U32" s="1" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="V32" s="1">
         <v>4.6</v>
       </c>
       <c r="W32" s="1" t="s">
-        <v>280</v>
+        <v>309</v>
       </c>
       <c r="X32" s="1">
         <v>4.0</v>
       </c>
       <c r="Y32" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="Z32" s="2"/>
+        <v>328</v>
+      </c>
+      <c r="Z32" s="6" t="s">
+        <v>329</v>
+      </c>
       <c r="AA32" s="2"/>
       <c r="AB32" s="2"/>
       <c r="AC32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="6">
+      <c r="A33" s="7">
         <v>32.0</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>298</v>
+      <c r="B33" s="7" t="s">
+        <v>330</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>299</v>
+        <v>331</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>300</v>
+        <v>332</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>301</v>
+        <v>333</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="P33" s="13" t="s">
-        <v>302</v>
-      </c>
-      <c r="Q33" s="13">
+        <v>95</v>
+      </c>
+      <c r="P33" s="14" t="s">
+        <v>334</v>
+      </c>
+      <c r="Q33" s="14">
         <v>25.054472694851</v>
       </c>
-      <c r="R33" s="13">
+      <c r="R33" s="14">
         <v>121.597933583479</v>
       </c>
       <c r="S33" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="T33" s="14" t="s">
-        <v>304</v>
+        <v>335</v>
+      </c>
+      <c r="T33" s="15" t="s">
+        <v>336</v>
       </c>
       <c r="U33" s="1" t="s">
-        <v>305</v>
+        <v>337</v>
       </c>
       <c r="V33" s="1">
         <v>4.6</v>
       </c>
       <c r="W33" s="1" t="s">
-        <v>306</v>
+        <v>338</v>
       </c>
       <c r="X33" s="1">
         <v>4.0</v>
       </c>
       <c r="Y33" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="Z33" s="2"/>
+        <v>339</v>
+      </c>
+      <c r="Z33" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="AA33" s="2"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
@@ -4088,152 +4273,157 @@
       <c r="A34" s="1">
         <v>33.0</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>308</v>
+      <c r="B34" s="7" t="s">
+        <v>341</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>309</v>
+        <v>342</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>300</v>
+        <v>332</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>311</v>
+        <v>344</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="P34" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="Q34" s="13">
+        <v>344</v>
+      </c>
+      <c r="P34" s="14" t="s">
+        <v>345</v>
+      </c>
+      <c r="Q34" s="14">
         <v>25.0543657837159</v>
       </c>
-      <c r="R34" s="13">
+      <c r="R34" s="14">
         <v>121.601560252277</v>
       </c>
       <c r="S34" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="T34" s="14" t="s">
-        <v>314</v>
+        <v>346</v>
+      </c>
+      <c r="T34" s="15" t="s">
+        <v>347</v>
       </c>
       <c r="U34" s="1" t="s">
-        <v>315</v>
+        <v>348</v>
       </c>
       <c r="V34" s="1">
         <v>4.6</v>
       </c>
       <c r="W34" s="1" t="s">
-        <v>306</v>
+        <v>338</v>
       </c>
       <c r="X34" s="1">
         <v>3.0</v>
       </c>
       <c r="Y34" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="Z34" s="2"/>
+        <v>349</v>
+      </c>
+      <c r="Z34" s="6" t="s">
+        <v>350</v>
+      </c>
       <c r="AA34" s="2"/>
       <c r="AB34" s="2"/>
       <c r="AC34" s="2"/>
     </row>
     <row r="35">
-      <c r="A35" s="6">
+      <c r="A35" s="7">
         <v>34.0</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>317</v>
+      <c r="B35" s="7" t="s">
+        <v>351</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>318</v>
+        <v>352</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>300</v>
+        <v>332</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>319</v>
+        <v>353</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="1" t="s">
-        <v>320</v>
+        <v>354</v>
       </c>
       <c r="K35" s="2"/>
       <c r="L35" s="1" t="s">
-        <v>320</v>
+        <v>354</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>320</v>
+        <v>354</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>320</v>
+        <v>354</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="P35" s="13" t="s">
-        <v>321</v>
-      </c>
-      <c r="Q35" s="13">
+        <v>123</v>
+      </c>
+      <c r="P35" s="14" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q35" s="14">
         <v>25.0547447224115</v>
       </c>
-      <c r="R35" s="13">
+      <c r="R35" s="14">
         <v>121.600253790755</v>
       </c>
       <c r="S35" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="T35" s="14" t="s">
-        <v>323</v>
+        <v>356</v>
+      </c>
+      <c r="T35" s="15" t="s">
+        <v>357</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>324</v>
+        <v>358</v>
       </c>
       <c r="V35" s="1">
         <v>4.9</v>
       </c>
       <c r="W35" s="1" t="s">
-        <v>306</v>
+        <v>338</v>
       </c>
       <c r="X35" s="1">
         <v>5.0</v>
       </c>
       <c r="Y35" s="1" t="s">
-        <v>325</v>
+        <v>359</v>
+      </c>
+      <c r="Z35" s="6" t="s">
+        <v>360</v>
       </c>
       <c r="AA35" s="2"/>
       <c r="AB35" s="2"/>
@@ -4243,152 +4433,156 @@
       <c r="A36" s="1">
         <v>35.0</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>326</v>
+      <c r="B36" s="7" t="s">
+        <v>361</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>327</v>
+        <v>362</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>329</v>
+        <v>364</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>330</v>
+        <v>365</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>330</v>
+        <v>365</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>331</v>
+        <v>366</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="1" t="s">
-        <v>331</v>
+        <v>366</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="P36" s="13" t="s">
-        <v>333</v>
-      </c>
-      <c r="Q36" s="13">
+        <v>367</v>
+      </c>
+      <c r="P36" s="14" t="s">
+        <v>368</v>
+      </c>
+      <c r="Q36" s="14">
         <v>24.9802196422302</v>
       </c>
-      <c r="R36" s="13">
+      <c r="R36" s="14">
         <v>121.55490196691</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="T36" s="14" t="s">
-        <v>335</v>
+        <v>369</v>
+      </c>
+      <c r="T36" s="15" t="s">
+        <v>370</v>
       </c>
       <c r="U36" s="1" t="s">
-        <v>305</v>
+        <v>337</v>
       </c>
       <c r="V36" s="1">
         <v>4.8</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="X36" s="1">
         <v>4.0</v>
       </c>
       <c r="Y36" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z36" s="2"/>
+        <v>372</v>
+      </c>
+      <c r="Z36" s="6" t="s">
+        <v>373</v>
+      </c>
       <c r="AA36" s="2"/>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2"/>
     </row>
     <row r="37">
-      <c r="A37" s="6">
+      <c r="A37" s="7">
         <v>36.0</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>338</v>
+      <c r="B37" s="7" t="s">
+        <v>374</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>339</v>
+        <v>375</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>340</v>
+        <v>376</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>340</v>
+        <v>376</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>340</v>
+        <v>376</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>340</v>
+        <v>376</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>340</v>
+        <v>376</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>340</v>
+        <v>376</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="P37" s="13" t="s">
-        <v>341</v>
-      </c>
-      <c r="Q37" s="13">
+        <v>376</v>
+      </c>
+      <c r="P37" s="14" t="s">
+        <v>377</v>
+      </c>
+      <c r="Q37" s="14">
         <v>24.9861372807182</v>
       </c>
-      <c r="R37" s="13">
+      <c r="R37" s="14">
         <v>121.570914328835</v>
       </c>
       <c r="S37" s="4" t="s">
-        <v>342</v>
-      </c>
-      <c r="T37" s="14" t="s">
-        <v>343</v>
+        <v>378</v>
+      </c>
+      <c r="T37" s="15" t="s">
+        <v>379</v>
       </c>
       <c r="U37" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V37" s="1">
         <v>4.7</v>
       </c>
       <c r="W37" s="1" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="X37" s="1">
         <v>5.0</v>
       </c>
       <c r="Y37" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="Z37" s="2"/>
+        <v>380</v>
+      </c>
+      <c r="Z37" s="6" t="s">
+        <v>381</v>
+      </c>
       <c r="AA37" s="2"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
@@ -4397,77 +4591,79 @@
       <c r="A38" s="1">
         <v>37.0</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>345</v>
+      <c r="B38" s="7" t="s">
+        <v>382</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>346</v>
+        <v>383</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>347</v>
+        <v>384</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="M38" s="2"/>
       <c r="N38" s="1" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="P38" s="13" t="s">
-        <v>349</v>
-      </c>
-      <c r="Q38" s="13">
+        <v>385</v>
+      </c>
+      <c r="P38" s="14" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q38" s="14">
         <v>24.9939153631141</v>
       </c>
-      <c r="R38" s="13">
+      <c r="R38" s="14">
         <v>121.545921750063</v>
       </c>
       <c r="S38" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="T38" s="14" t="s">
-        <v>351</v>
+        <v>387</v>
+      </c>
+      <c r="T38" s="15" t="s">
+        <v>388</v>
       </c>
       <c r="U38" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="V38" s="1">
         <v>4.5</v>
       </c>
       <c r="W38" s="1" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="X38" s="1">
         <v>4.0</v>
       </c>
       <c r="Y38" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="Z38" s="2"/>
+        <v>389</v>
+      </c>
+      <c r="Z38" s="6" t="s">
+        <v>390</v>
+      </c>
       <c r="AA38" s="2"/>
       <c r="AB38" s="2"/>
       <c r="AC38" s="2"/>
@@ -4527,122 +4723,122 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="s">
-        <v>353</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>354</v>
-      </c>
-      <c r="C1" s="15" t="s">
+      <c r="A1" s="16" t="s">
+        <v>391</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="15" t="s">
-        <v>355</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>356</v>
-      </c>
-      <c r="G1" s="15" t="s">
+      <c r="E1" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>394</v>
+      </c>
+      <c r="G1" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>357</v>
-      </c>
-      <c r="C2" s="16">
+      <c r="A2" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="C2" s="17">
         <v>121.523577</v>
       </c>
-      <c r="D2" s="16">
+      <c r="D2" s="17">
         <v>25.050734</v>
       </c>
-      <c r="E2" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="15" t="s">
-        <v>359</v>
+      <c r="E2" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="F2" s="18"/>
+      <c r="G2" s="16" t="s">
+        <v>397</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>360</v>
+        <v>398</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>361</v>
-      </c>
-      <c r="C3" s="16">
+      <c r="A3" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="C3" s="17">
         <v>121.552515</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="17">
         <v>25.04379</v>
       </c>
-      <c r="E3" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="F3" s="17"/>
-      <c r="G3" s="15" t="s">
-        <v>362</v>
+      <c r="E3" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3" s="16" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="C4" s="16">
+      <c r="A4" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>401</v>
+      </c>
+      <c r="C4" s="17">
         <v>121.521245</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="17">
         <v>25.05093</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>365</v>
+      <c r="E4" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>366</v>
-      </c>
-      <c r="C5" s="16">
+      <c r="A5" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>404</v>
+      </c>
+      <c r="C5" s="17">
         <v>121.520531</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="17">
         <v>25.049479</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>367</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>368</v>
+      <c r="E5" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>405</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="6">
       <c r="N6" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add images and add snackbar msg English version
</commit_message>
<xml_diff>
--- a/public/data/Taipei_Retro_Cafe.xlsx
+++ b/public/data/Taipei_Retro_Cafe.xlsx
@@ -284,7 +284,7 @@
     <t>No. 302, Wenlin Rd, Shilin District</t>
   </si>
   <si>
-    <t>Retro Station is a charming old-house café near Shipai Station. The warm vintage design, handcrafted lattes, and brunch options make it a great place to slow down and relax.</t>
+    <t>Orange Cafe, located near Taipei's Shilin MRT Station, offers a diverse coffee selection, from Italian to specialty lattes, catering to all tastes. The comfortable cafe features large second-floor windows for MRT train viewing and a relaxed third-floor outdoor area. It provides free Wi-Fi and some power outlets (NT$30 fee). With no dining time limit, it's ideal for reading, working, or social gatherings.</t>
   </si>
   <si>
     <t>幻猻家珈琲</t>
@@ -407,7 +407,7 @@
     <t>No. 1, Alley 6, Lane 147, Section 2, Minsheng E Rd, Zhongshan District</t>
   </si>
   <si>
-    <t>Combining Taiwanese old-school charm with specialty brews, this café serves single-origin coffee in a cozy, low-key setting that invites you to linger.</t>
+    <t>This eye-catching, retro royal-blue cafe, with its black and white floral tiles, offers an exotic, English-style ambiance. Perfect for a "fake abroad" experience. You can dine in or take away. The owner transitioned from finance. The cozy interior features a window bar and three small tables, ideal for office workers grabbing takeaway coffee before work.</t>
   </si>
   <si>
     <t>二會咖啡廳</t>
@@ -752,7 +752,7 @@
     <t>No. 10, Lane 73, Tong'an St, Zhongzheng District</t>
   </si>
   <si>
-    <t>This small café packs a lot of character. Retro decor and warm smiles welcome you at the door. Their coffee is as rich in flavor as the space is in charm. It’s a space to sit back, sip slowly, and enjoy the moment.</t>
+    <t>WANGXIANG is a coffee shop blending Eastern philosophy with modern minimalism, nestled quietly in the city. Its wood tones and minimalist design create a serene atmosphere, fostering inner balance. Specializing in pour-over specialty coffee and seasonal desserts, WANGXIANG meticulously crafts every detail from bean to brew. It's a place to slow down and reconnect with life's finer details, whether you're reading, creating, or chatting with friends.</t>
   </si>
   <si>
     <t>4F劇場咖啡</t>
@@ -1094,7 +1094,7 @@
     <t>1F, No. 26, Lane 178, Section 2, Nangang Rd, Nangang District</t>
   </si>
   <si>
-    <t>Designed with a retro spirit, this café highlights Taiwan’s cultural past. The baristas are skilled in pour-over technique, and the drinks are beautifully balanced. It’s a space that feels both curated and homey.</t>
+    <t>Tian Ye Coffee is a Japanese-style cafe that blends a retro atmosphere with exquisite coffee. The interior features primarily wooden decor, creating a warm and comfortable ambiance. It offers unlimited seating time and power outlets, making it ideal for longer stays. The menu includes various coffees, floral teas, and light meals, paired with handmade desserts like chocolate cake and tiramisu, which are highly popular among customers.</t>
   </si>
   <si>
     <t>咖啡喫茶 枝音</t>
@@ -1157,7 +1157,7 @@
     <t>1F, No. 1, Lane 69, Section 2, Muxin Rd, Wenshan District</t>
   </si>
   <si>
-    <t>This space is a tribute to quiet beauty. Guests sip thoughtfully made drinks surrounded by retro details. It’s calm, familiar, and softly lit. The kind of place that becomes a habit.</t>
+    <t>CCIP &amp; CAFE is a hidden spot merging art, culture, and coffee. This old house retains its charm with vintage decor, offering a warm, cozy atmosphere. Enjoy unlimited seating and power outlets. They host diverse events like starlight cinema and concerts, providing unique cultural experiences. It's more than a cafe; it's a hub of creativity and freedom.</t>
   </si>
   <si>
     <t>聞山咖啡</t>
@@ -1184,7 +1184,7 @@
     <t>No. 19, Jingzhong St, Wenshan District</t>
   </si>
   <si>
-    <t>Sunlight spills over the vintage tiles and weathered wood of this serene café. Their coffee is balanced and aromatic. Time seems to move differently here. Every visit feels like a treat.</t>
+    <t>Since 1985, "Wen Shan Coffee" has upheld its commitment to traditional roasting, pour-over methods, and homemade desserts. Its interior blends Japanese and Taiwanese elements, creating a warm ambiance. Despite digitalization, Wen Shan Coffee remains dedicated to handcraftsmanship and personal touch, solidifying its status as a local cultural landmark through unwavering quality and tradition.</t>
   </si>
   <si>
     <t>地區</t>
@@ -1299,7 +1299,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1329,6 +1329,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -1737,7 +1740,7 @@
         <v>37</v>
       </c>
       <c r="X2" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y2" s="5" t="s">
         <v>38</v>
@@ -2164,7 +2167,7 @@
       <c r="Y7" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="Z7" s="6" t="s">
+      <c r="Z7" s="10" t="s">
         <v>90</v>
       </c>
       <c r="AA7" s="2"/>
@@ -2491,7 +2494,7 @@
       <c r="Y11" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="Z11" s="6" t="s">
+      <c r="Z11" s="10" t="s">
         <v>131</v>
       </c>
       <c r="AA11" s="2"/>
@@ -2814,7 +2817,7 @@
         <v>157</v>
       </c>
       <c r="X15" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y15" s="5" t="s">
         <v>167</v>
@@ -2893,7 +2896,7 @@
         <v>157</v>
       </c>
       <c r="X16" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y16" s="5" t="s">
         <v>177</v>
@@ -2969,7 +2972,7 @@
         <v>189</v>
       </c>
       <c r="X17" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y17" s="5" t="s">
         <v>190</v>
@@ -3216,7 +3219,7 @@
         <v>100</v>
       </c>
       <c r="X20" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y20" s="1" t="s">
         <v>214</v>
@@ -3445,7 +3448,7 @@
       <c r="S23" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="T23" s="10" t="s">
+      <c r="T23" s="11" t="s">
         <v>242</v>
       </c>
       <c r="U23" s="1" t="s">
@@ -3458,12 +3461,12 @@
         <v>244</v>
       </c>
       <c r="X23" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y23" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="Z23" s="6" t="s">
+      <c r="Z23" s="10" t="s">
         <v>246</v>
       </c>
       <c r="AB23" s="2"/>
@@ -3527,7 +3530,7 @@
       <c r="S24" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="T24" s="11" t="s">
+      <c r="T24" s="12" t="s">
         <v>251</v>
       </c>
       <c r="U24" s="1" t="s">
@@ -3540,7 +3543,7 @@
         <v>244</v>
       </c>
       <c r="X24" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y24" s="5" t="s">
         <v>252</v>
@@ -3603,7 +3606,7 @@
       <c r="S25" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="T25" s="12" t="s">
+      <c r="T25" s="13" t="s">
         <v>259</v>
       </c>
       <c r="U25" s="1" t="s">
@@ -3616,7 +3619,7 @@
         <v>244</v>
       </c>
       <c r="X25" s="1">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="Y25" s="5" t="s">
         <v>261</v>
@@ -3684,7 +3687,7 @@
       <c r="S26" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="T26" s="11" t="s">
+      <c r="T26" s="12" t="s">
         <v>269</v>
       </c>
       <c r="U26" s="1" t="s">
@@ -3762,7 +3765,7 @@
       <c r="S27" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="T27" s="10" t="s">
+      <c r="T27" s="11" t="s">
         <v>279</v>
       </c>
       <c r="U27" s="1" t="s">
@@ -3843,7 +3846,7 @@
       <c r="S28" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="T28" s="12" t="s">
+      <c r="T28" s="13" t="s">
         <v>289</v>
       </c>
       <c r="U28" s="1" t="s">
@@ -3921,7 +3924,7 @@
       <c r="R29" s="1">
         <v>121.553897808577</v>
       </c>
-      <c r="S29" s="13" t="s">
+      <c r="S29" s="14" t="s">
         <v>296</v>
       </c>
       <c r="T29" s="9" t="s">
@@ -4080,7 +4083,7 @@
       <c r="R31" s="2">
         <v>121.563086959166</v>
       </c>
-      <c r="S31" s="13" t="s">
+      <c r="S31" s="14" t="s">
         <v>316</v>
       </c>
       <c r="T31" s="9" t="s">
@@ -4158,7 +4161,7 @@
       <c r="R32" s="1">
         <v>121.563566049973</v>
       </c>
-      <c r="S32" s="13" t="s">
+      <c r="S32" s="14" t="s">
         <v>326</v>
       </c>
       <c r="T32" s="9" t="s">
@@ -4232,19 +4235,19 @@
       <c r="O33" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="P33" s="14" t="s">
+      <c r="P33" s="15" t="s">
         <v>334</v>
       </c>
-      <c r="Q33" s="14">
+      <c r="Q33" s="15">
         <v>25.054472694851</v>
       </c>
-      <c r="R33" s="14">
+      <c r="R33" s="15">
         <v>121.597933583479</v>
       </c>
       <c r="S33" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="T33" s="15" t="s">
+      <c r="T33" s="16" t="s">
         <v>336</v>
       </c>
       <c r="U33" s="1" t="s">
@@ -4313,19 +4316,19 @@
       <c r="O34" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="P34" s="14" t="s">
+      <c r="P34" s="15" t="s">
         <v>345</v>
       </c>
-      <c r="Q34" s="14">
+      <c r="Q34" s="15">
         <v>25.0543657837159</v>
       </c>
-      <c r="R34" s="14">
+      <c r="R34" s="15">
         <v>121.601560252277</v>
       </c>
       <c r="S34" s="4" t="s">
         <v>346</v>
       </c>
-      <c r="T34" s="15" t="s">
+      <c r="T34" s="16" t="s">
         <v>347</v>
       </c>
       <c r="U34" s="1" t="s">
@@ -4392,19 +4395,19 @@
       <c r="O35" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="P35" s="14" t="s">
+      <c r="P35" s="15" t="s">
         <v>355</v>
       </c>
-      <c r="Q35" s="14">
+      <c r="Q35" s="15">
         <v>25.0547447224115</v>
       </c>
-      <c r="R35" s="14">
+      <c r="R35" s="15">
         <v>121.600253790755</v>
       </c>
       <c r="S35" s="4" t="s">
         <v>356</v>
       </c>
-      <c r="T35" s="15" t="s">
+      <c r="T35" s="16" t="s">
         <v>357</v>
       </c>
       <c r="U35" s="1" t="s">
@@ -4422,7 +4425,7 @@
       <c r="Y35" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="Z35" s="6" t="s">
+      <c r="Z35" s="10" t="s">
         <v>360</v>
       </c>
       <c r="AA35" s="2"/>
@@ -4471,19 +4474,19 @@
       <c r="O36" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="P36" s="14" t="s">
+      <c r="P36" s="15" t="s">
         <v>368</v>
       </c>
-      <c r="Q36" s="14">
+      <c r="Q36" s="15">
         <v>24.9802196422302</v>
       </c>
-      <c r="R36" s="14">
+      <c r="R36" s="15">
         <v>121.55490196691</v>
       </c>
       <c r="S36" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="T36" s="15" t="s">
+      <c r="T36" s="16" t="s">
         <v>370</v>
       </c>
       <c r="U36" s="1" t="s">
@@ -4550,19 +4553,19 @@
       <c r="O37" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="P37" s="14" t="s">
+      <c r="P37" s="15" t="s">
         <v>377</v>
       </c>
-      <c r="Q37" s="14">
+      <c r="Q37" s="15">
         <v>24.9861372807182</v>
       </c>
-      <c r="R37" s="14">
+      <c r="R37" s="15">
         <v>121.570914328835</v>
       </c>
       <c r="S37" s="4" t="s">
         <v>378</v>
       </c>
-      <c r="T37" s="15" t="s">
+      <c r="T37" s="16" t="s">
         <v>379</v>
       </c>
       <c r="U37" s="1" t="s">
@@ -4580,7 +4583,7 @@
       <c r="Y37" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="Z37" s="6" t="s">
+      <c r="Z37" s="10" t="s">
         <v>381</v>
       </c>
       <c r="AA37" s="2"/>
@@ -4631,19 +4634,19 @@
       <c r="O38" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="P38" s="14" t="s">
+      <c r="P38" s="15" t="s">
         <v>386</v>
       </c>
-      <c r="Q38" s="14">
+      <c r="Q38" s="15">
         <v>24.9939153631141</v>
       </c>
-      <c r="R38" s="14">
+      <c r="R38" s="15">
         <v>121.545921750063</v>
       </c>
       <c r="S38" s="4" t="s">
         <v>387</v>
       </c>
-      <c r="T38" s="15" t="s">
+      <c r="T38" s="16" t="s">
         <v>388</v>
       </c>
       <c r="U38" s="1" t="s">
@@ -4661,7 +4664,7 @@
       <c r="Y38" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="Z38" s="6" t="s">
+      <c r="Z38" s="10" t="s">
         <v>390</v>
       </c>
       <c r="AA38" s="2"/>
@@ -4723,46 +4726,46 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>391</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="17" t="s">
         <v>392</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="17" t="s">
         <v>393</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="17" t="s">
         <v>394</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="17" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>395</v>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="18">
         <v>121.523577</v>
       </c>
-      <c r="D2" s="17">
+      <c r="D2" s="18">
         <v>25.050734</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="16" t="s">
+      <c r="F2" s="19"/>
+      <c r="G2" s="17" t="s">
         <v>397</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -4770,69 +4773,69 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="17" t="s">
         <v>264</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>399</v>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="18">
         <v>121.552515</v>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="18">
         <v>25.04379</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="16" t="s">
+      <c r="F3" s="19"/>
+      <c r="G3" s="17" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>401</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="18">
         <v>121.521245</v>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="18">
         <v>25.05093</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="17" t="s">
         <v>402</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="17" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>404</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="18">
         <v>121.520531</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="18">
         <v>25.049479</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="17" t="s">
         <v>396</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>405</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>406</v>
       </c>
     </row>

</xml_diff>